<commit_message>
Link on provider name
</commit_message>
<xml_diff>
--- a/data/vendors-live.xlsx
+++ b/data/vendors-live.xlsx
@@ -2305,7 +2305,7 @@
         <v>157</v>
       </c>
       <c r="F26" t="s">
-        <v>188</v>
+        <v>75</v>
       </c>
       <c r="G26">
         <v>40</v>
@@ -2386,7 +2386,7 @@
         <v>164</v>
       </c>
       <c r="F29" t="s">
-        <v>188</v>
+        <v>88</v>
       </c>
       <c r="G29">
         <v>1250</v>

</xml_diff>